<commit_message>
Docs : Mise à jour initialisation du sprint-backlog
</commit_message>
<xml_diff>
--- a/docs/Cadrage projet/sprint-backlog.xlsx
+++ b/docs/Cadrage projet/sprint-backlog.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nastry Gamer\Desktop\Programation\Cours\IPSSI_APOCAL_KIT\docs\Cadrage projet\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nastry Gamer\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8577203-914B-4734-A5DC-CCF4226200C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{250ACE72-3FC4-47D8-91AB-62F318530F02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3465" yWindow="3465" windowWidth="38700" windowHeight="15345" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Garde" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="141">
   <si>
     <t>A</t>
   </si>
@@ -59,9 +59,6 @@
     <t>Membres</t>
   </si>
   <si>
-    <t>[ Prénoms NOMS, séparés par virgule ]</t>
-  </si>
-  <si>
     <t>Sprint concerné</t>
   </si>
   <si>
@@ -98,9 +95,6 @@
     <t>Date</t>
   </si>
   <si>
-    <t>Lundi [JJ/MM/AAAA], 14h00 à 18h00 (4 h)</t>
-  </si>
-  <si>
     <t>Équipe (n personnes)</t>
   </si>
   <si>
@@ -182,9 +176,6 @@
     <t>Modèle User Django (extension AbstractUser) + migration</t>
   </si>
   <si>
-    <t>[ Prénom ]</t>
-  </si>
-  <si>
     <t>Todo</t>
   </si>
   <si>
@@ -308,9 +299,6 @@
     <t>14h00, Début sprint</t>
   </si>
   <si>
-    <t>[à compléter]</t>
-  </si>
-  <si>
     <t>Début sprint, toutes tâches en Todo</t>
   </si>
   <si>
@@ -435,6 +423,30 @@
   </si>
   <si>
     <t>Prof</t>
+  </si>
+  <si>
+    <t>Sebastien</t>
+  </si>
+  <si>
+    <t>Syphax</t>
+  </si>
+  <si>
+    <t>Jacqueline</t>
+  </si>
+  <si>
+    <t>Killian</t>
+  </si>
+  <si>
+    <t>Moussa</t>
+  </si>
+  <si>
+    <t>Amine</t>
+  </si>
+  <si>
+    <t>Lundi 29/06/2026, 14h00 à 18h00 (4 h)</t>
+  </si>
+  <si>
+    <t>Tristan DZIOCH · Sebastien GERARD · Syphax ALILI · Killian MARTINS · Amine TALEB · Jacqueline MAPENZI · Moussa DIOP</t>
   </si>
 </sst>
 </file>
@@ -1088,7 +1100,7 @@
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="60" customWidth="1"/>
+    <col min="3" max="3" width="107.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
@@ -1114,49 +1126,49 @@
         <v>10</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>11</v>
+        <v>140</v>
       </c>
     </row>
     <row r="7" spans="2:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="8" spans="2:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
     </row>
     <row r="9" spans="2:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="10" spans="2:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B12" s="12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B13" s="7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -1179,150 +1191,150 @@
   <sheetData>
     <row r="1" spans="1:2" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A1" s="13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="15" t="s">
         <v>21</v>
-      </c>
-      <c r="B5" s="15" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>24</v>
+        <v>139</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="16" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="17" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="B19" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="C19" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="B19" s="18" t="s">
+      <c r="D19" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="C19" s="18" t="s">
+      <c r="E19" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="D19" s="18" t="s">
+      <c r="F19" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="E19" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="F19" s="18" t="s">
-        <v>48</v>
-      </c>
       <c r="G19" s="18" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="B20" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="C20" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="B20" s="19" t="s">
-        <v>50</v>
-      </c>
-      <c r="C20" s="20" t="s">
-        <v>51</v>
-      </c>
       <c r="D20" s="20" t="s">
-        <v>52</v>
+        <v>135</v>
       </c>
       <c r="E20" s="21">
         <v>1</v>
@@ -1331,21 +1343,21 @@
         <v>1</v>
       </c>
       <c r="G20" s="20" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="19" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C21" s="20" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D21" s="20" t="s">
-        <v>52</v>
+        <v>138</v>
       </c>
       <c r="E21" s="21">
         <v>2</v>
@@ -1354,21 +1366,21 @@
         <v>2</v>
       </c>
       <c r="G21" s="20" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="19" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C22" s="20" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D22" s="20" t="s">
-        <v>52</v>
+        <v>137</v>
       </c>
       <c r="E22" s="21">
         <v>3</v>
@@ -1377,21 +1389,21 @@
         <v>3</v>
       </c>
       <c r="G22" s="20" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="19" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C23" s="20" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D23" s="20" t="s">
-        <v>52</v>
+        <v>133</v>
       </c>
       <c r="E23" s="21">
         <v>1</v>
@@ -1400,21 +1412,21 @@
         <v>1</v>
       </c>
       <c r="G23" s="20" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="22" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B24" s="22" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C24" s="23" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D24" s="23" t="s">
-        <v>52</v>
+        <v>135</v>
       </c>
       <c r="E24" s="24">
         <v>1</v>
@@ -1423,21 +1435,21 @@
         <v>1</v>
       </c>
       <c r="G24" s="23" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="22" t="s">
+        <v>57</v>
+      </c>
+      <c r="B25" s="22" t="s">
         <v>60</v>
       </c>
-      <c r="B25" s="22" t="s">
-        <v>63</v>
-      </c>
       <c r="C25" s="23" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D25" s="23" t="s">
-        <v>52</v>
+        <v>136</v>
       </c>
       <c r="E25" s="24">
         <v>3</v>
@@ -1446,21 +1458,21 @@
         <v>3</v>
       </c>
       <c r="G25" s="23" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="22" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B26" s="22" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C26" s="23" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="D26" s="23" t="s">
-        <v>52</v>
+        <v>135</v>
       </c>
       <c r="E26" s="24">
         <v>1</v>
@@ -1469,21 +1481,21 @@
         <v>1</v>
       </c>
       <c r="G26" s="23" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="22" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B27" s="22" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C27" s="23" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D27" s="23" t="s">
-        <v>52</v>
+        <v>134</v>
       </c>
       <c r="E27" s="24">
         <v>3</v>
@@ -1492,21 +1504,21 @@
         <v>3</v>
       </c>
       <c r="G27" s="23" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="22" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B28" s="22" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C28" s="23" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D28" s="23" t="s">
-        <v>52</v>
+        <v>133</v>
       </c>
       <c r="E28" s="24">
         <v>1</v>
@@ -1515,29 +1527,29 @@
         <v>1</v>
       </c>
       <c r="G28" s="23" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="25"/>
       <c r="B29" s="25"/>
       <c r="C29" s="26" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="D29" s="26"/>
       <c r="E29" s="27"/>
       <c r="F29" s="27"/>
       <c r="G29" s="26" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="28" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B30" s="29"/>
       <c r="C30" s="30" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="D30" s="29"/>
       <c r="E30" s="28">
@@ -1550,39 +1562,39 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="31" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="32" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="17" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="16" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -1603,165 +1615,175 @@
   <sheetData>
     <row r="1" spans="1:5" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A1" s="13" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>87</v>
+      </c>
+      <c r="D7" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="E7" s="18" t="s">
         <v>89</v>
-      </c>
-      <c r="C7" s="18" t="s">
-        <v>90</v>
-      </c>
-      <c r="D7" s="18" t="s">
-        <v>91</v>
-      </c>
-      <c r="E7" s="18" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="33" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B8" s="34">
         <v>16</v>
       </c>
-      <c r="C8" s="34" t="s">
-        <v>94</v>
-      </c>
-      <c r="D8" s="34"/>
+      <c r="C8" s="34">
+        <v>16</v>
+      </c>
+      <c r="D8" s="34">
+        <v>0</v>
+      </c>
       <c r="E8" s="15" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="33" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B9" s="34">
         <v>12</v>
       </c>
-      <c r="C9" s="34" t="s">
-        <v>94</v>
-      </c>
-      <c r="D9" s="34"/>
+      <c r="C9" s="34">
+        <v>13</v>
+      </c>
+      <c r="D9" s="34">
+        <v>1</v>
+      </c>
       <c r="E9" s="15" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="33" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="B10" s="34">
         <v>8</v>
       </c>
-      <c r="C10" s="34" t="s">
-        <v>94</v>
-      </c>
-      <c r="D10" s="34"/>
+      <c r="C10" s="34">
+        <v>8</v>
+      </c>
+      <c r="D10" s="34">
+        <v>0</v>
+      </c>
       <c r="E10" s="15" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="33" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="B11" s="34">
         <v>4</v>
       </c>
-      <c r="C11" s="34" t="s">
-        <v>94</v>
-      </c>
-      <c r="D11" s="34"/>
+      <c r="C11" s="34">
+        <v>3</v>
+      </c>
+      <c r="D11" s="34">
+        <v>-1</v>
+      </c>
       <c r="E11" s="15" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="33" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="B12" s="34">
         <v>0</v>
       </c>
-      <c r="C12" s="34" t="s">
-        <v>94</v>
-      </c>
-      <c r="D12" s="34"/>
+      <c r="C12" s="34">
+        <v>1</v>
+      </c>
+      <c r="D12" s="34">
+        <v>1</v>
+      </c>
       <c r="E12" s="15" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="16" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="32" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="16" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="17" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -1782,113 +1804,113 @@
   <sheetData>
     <row r="2" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B2" s="2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B3" s="9" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="18"/>
       <c r="B5" s="18" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="D5" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="35" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C6" s="36" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="D6" s="35"/>
     </row>
     <row r="7" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="35" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="C7" s="36" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="D7" s="35"/>
     </row>
     <row r="8" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="35" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="C8" s="36" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="D8" s="35"/>
     </row>
     <row r="9" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="35" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="C9" s="36" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="D9" s="35"/>
     </row>
     <row r="10" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="35" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C10" s="36" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="D10" s="35"/>
     </row>
     <row r="11" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="35" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C11" s="36" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="D11" s="35"/>
     </row>
     <row r="12" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="35" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C12" s="36" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="D12" s="35"/>
     </row>
     <row r="13" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="35" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="C13" s="36" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="D13" s="35"/>
     </row>
     <row r="14" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="35" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C14" s="36" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="D14" s="35"/>
     </row>
     <row r="15" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="35" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C15" s="36" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="D15" s="35"/>
     </row>

</xml_diff>